<commit_message>
Updated Financial Policies and Procedures
</commit_message>
<xml_diff>
--- a/Finance Policies & Procedures/Budget Templates/USDA Sub Activity Template 2025-05.xlsx
+++ b/Finance Policies & Procedures/Budget Templates/USDA Sub Activity Template 2025-05.xlsx
@@ -13495,8 +13495,8 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003206C8355D678A459F2EF8957171B231" ma:contentTypeVersion="18" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="c89dbf13fad0b1343cd41b5338c7e736">
-  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f2466082-b6bf-4153-98c3-3c41e85fda18" xmlns:ns3="dc808d36-874f-4b27-aec2-2fd649817929" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bd4a7335f490c5a41276d1fccfad81ee" ns2:_="" ns3:_="">
+<ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x0101003206C8355D678A459F2EF8957171B231" ma:contentTypeVersion="19" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="a5577d833b9f28dcc6be37a04859b9a8">
+  <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="f2466082-b6bf-4153-98c3-3c41e85fda18" xmlns:ns3="dc808d36-874f-4b27-aec2-2fd649817929" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="ae50cb7862d574a2d96b6910b4abdc85" ns2:_="" ns3:_="">
     <xsd:import namespace="f2466082-b6bf-4153-98c3-3c41e85fda18"/>
     <xsd:import namespace="dc808d36-874f-4b27-aec2-2fd649817929"/>
     <xsd:element name="properties">
@@ -13522,6 +13522,7 @@
                 <xsd:element ref="ns3:TaxCatchAll" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceSearchProperties" minOccurs="0"/>
                 <xsd:element ref="ns2:MediaServiceObjectDetectorVersions" minOccurs="0"/>
+                <xsd:element ref="ns2:MediaServiceBillingMetadata" minOccurs="0"/>
               </xsd:all>
             </xsd:complexType>
           </xsd:element>
@@ -13606,6 +13607,11 @@
     <xsd:element name="MediaServiceObjectDetectorVersions" ma:index="25" nillable="true" ma:displayName="MediaServiceObjectDetectorVersions" ma:hidden="true" ma:indexed="true" ma:internalName="MediaServiceObjectDetectorVersions" ma:readOnly="true">
       <xsd:simpleType>
         <xsd:restriction base="dms:Text"/>
+      </xsd:simpleType>
+    </xsd:element>
+    <xsd:element name="MediaServiceBillingMetadata" ma:index="26" nillable="true" ma:displayName="MediaServiceBillingMetadata" ma:hidden="true" ma:internalName="MediaServiceBillingMetadata" ma:readOnly="true">
+      <xsd:simpleType>
+        <xsd:restriction base="dms:Note"/>
       </xsd:simpleType>
     </xsd:element>
   </xsd:schema>
@@ -13769,20 +13775,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D876BE8F-E597-49DF-AB8F-1CD0D715DA59}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="f2466082-b6bf-4153-98c3-3c41e85fda18"/>
-    <ds:schemaRef ds:uri="dc808d36-874f-4b27-aec2-2fd649817929"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{0D50F81B-A32C-49C0-9F3F-0C7838183AA5}"/>
 </file>
</xml_diff>